<commit_message>
REV9: mating plug wording (WeGo inquiry)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QuQ76tLZcwBitJJSmeNKWm
</commit_message>
<xml_diff>
--- a/out/SBOX_REV9_BOM.xlsx
+++ b/out/SBOX_REV9_BOM.xlsx
@@ -3294,32 +3294,15 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9.5"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">동봉 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9.5"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9.5"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">핀 항공 플러그 </t>
+      <t xml:space="preserve">: 4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">핀 항공 메이팅 플러그 </t>
     </r>
     <r>
       <rPr>
@@ -3366,7 +3349,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">납땜 제작</t>
+    <t xml:space="preserve">플러그 규격 위고 확인</t>
   </si>
   <si>
     <t xml:space="preserve">H1</t>
@@ -3378,24 +3361,24 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">위고 제작 요청 중 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9.5"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9.5"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">불가 시 </t>
+      <t xml:space="preserve">확보 방법 위고 문의 중 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">구매 또는 </t>
     </r>
     <r>
       <rPr>
@@ -3414,6 +3397,15 @@
       </rPr>
       <t xml:space="preserve">납땜</t>
     </r>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">CABLE</t>
@@ -4284,17 +4276,34 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">핀 항공 플러그 모델</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9.5"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">동봉 플러그에 케이블 납땜 → </t>
+      <t xml:space="preserve">핀 항공 메이팅 플러그 규격</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">위고 문의 → 플러그</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.5"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">케이블 확보 후 </t>
     </r>
     <r>
       <rPr>

</xml_diff>